<commit_message>
Record Transitions queue ID 13519270 in teams.json
WLS confirmed 13519270 is the Transitions queue. Updates F-13, the
README and the HTML summary to match; the v2 workbook is rebuilt from
the same fetch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017uf8FUtnaXSoM3iiDFsscT
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit_v2.xlsx
+++ b/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit_v2.xlsx
@@ -11079,22 +11079,22 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Team check 1 (queue): 26 of 31 Create task actions set queue ID 13519270, which this audit treats as the Transitions queue. The other 5 are the Go-Live Execution actions (see the queue finding). The API cannot return queue names, so it is not confirmed that 13519270 is the queue named "Transitions". The 4 "Marketing | Create Marketing Proposal" actions (Pre-Launch Setup, Steps 8-11) also use 13519270 although they are assigned to Brock Hegr, Sarah Schlosberg and Mohammad Abudahab. VERIFIED (config).</t>
+          <t>Team check 1 (queue): 26 of 31 Create task actions set queue ID 13519270. WLS confirmed on 2026-10-06 that this is the "Transitions" queue, and it is now in teams.json. The other 5 are the Go-Live Execution actions, which set no queue (see the queue finding). The 4 "Marketing | Create Marketing Proposal" actions (Pre-Launch Setup, Steps 8-11) also use the Transitions queue, although they are assigned to Brock Hegr, Sarah Schlosberg and Mohammad Abudahab. VERIFIED (config); queue name confirmed by WLS.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Config queue_id on all 31 Create task actions; teams.json has no queue_ids for Transitions (CS Ops "Ops Tasks" is 13519269).</t>
+          <t>Config queue_id on all 31 Create task actions; teams.json Transitions queue_ids = ["13519270"].</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>If 13519270 is not the Transitions queue, every task is outside the team's queue. Marketing proposal tasks in the Transitions queue may not be seen by the marketing managers they are assigned to.</t>
+          <t>Marketing proposal tasks in the Transitions queue may not be seen by the marketing managers they are assigned to.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>In HubSpot (Tasks &gt; Queues), confirm that queue ID 13519270 is "Transitions", then add it to teams.json. Confirm the marketing proposal tasks are meant to sit in the Transitions queue.</t>
+          <t>Confirm the marketing proposal tasks are meant to sit in the Transitions queue.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">

</xml_diff>